<commit_message>
Actions and Project Reports Impleted
</commit_message>
<xml_diff>
--- a/BCTGovernanceOne.xlsx
+++ b/BCTGovernanceOne.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\ProjectGovernance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE9C8121-52EF-459F-9E27-A5942531465C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A512FEFC-EBBC-45D8-A3D9-1C17A1DF65D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="897" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="897" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="22" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <externalReference r:id="rId23"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Changes!$A$1:$C$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Changes!$A$1:$C$152</definedName>
     <definedName name="Phases">'[1]Hide '!$B$26:$B$31</definedName>
     <definedName name="Source">'[1]Hide '!$B$38:$B$43</definedName>
   </definedNames>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1422" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="783">
   <si>
     <t>Project Type</t>
   </si>
@@ -2427,9 +2427,6 @@
     <t>In All Pages, Project Dashboard should be renamed as Delivery Status Report &amp; Project Performance Report</t>
   </si>
   <si>
-    <t xml:space="preserve">Action Flow - </t>
-  </si>
-  <si>
     <t>New Action Creation / View Page from Left Menu</t>
   </si>
   <si>
@@ -2482,6 +2479,30 @@
   </si>
   <si>
     <t>Onboarding of All Projects</t>
+  </si>
+  <si>
+    <t>Provision to view Oracle projects that are not mapped in Governance projects</t>
+  </si>
+  <si>
+    <t>In PM My Summary, we have 20 projects, but Project Health is declared for 5. Show remaining 15 as not assessed</t>
+  </si>
+  <si>
+    <t>Action Flow - When actions are created from Report pages, the level section combo and value combo should disabled. Action can be created only for that context</t>
+  </si>
+  <si>
+    <t>DE Approval</t>
+  </si>
+  <si>
+    <t>Report Project Status</t>
+  </si>
+  <si>
+    <t>DE Assessment</t>
+  </si>
+  <si>
+    <t>DE Findings</t>
+  </si>
+  <si>
+    <t>DE Project Approval</t>
   </si>
 </sst>
 </file>
@@ -3504,7 +3525,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="274">
+  <cellXfs count="275">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
@@ -3913,6 +3934,10 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="4" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3925,18 +3950,72 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3944,63 +4023,9 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4029,10 +4054,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Excel Built-in Normal" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -4508,143 +4532,143 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18">
-      <c r="A1" s="273" t="s">
+      <c r="A1" s="217" t="s">
+        <v>761</v>
+      </c>
+      <c r="B1" s="217" t="s">
         <v>762</v>
       </c>
-      <c r="B1" s="273" t="s">
+      <c r="C1" s="217" t="s">
         <v>763</v>
       </c>
-      <c r="C1" s="273" t="s">
-        <v>764</v>
-      </c>
-      <c r="D1" s="273" t="s">
+      <c r="D1" s="217" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="33" t="s">
-        <v>765</v>
-      </c>
-      <c r="B2" s="270">
+        <v>764</v>
+      </c>
+      <c r="B2" s="214">
         <v>46220</v>
       </c>
-      <c r="C2" s="270">
+      <c r="C2" s="214">
         <v>46227</v>
       </c>
-      <c r="D2" s="271" t="s">
+      <c r="D2" s="215" t="s">
         <v>559</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="33" t="s">
-        <v>766</v>
-      </c>
-      <c r="B3" s="270">
+        <v>765</v>
+      </c>
+      <c r="B3" s="214">
         <v>46227</v>
       </c>
-      <c r="C3" s="270">
+      <c r="C3" s="214">
         <v>46241</v>
       </c>
-      <c r="D3" s="271" t="s">
+      <c r="D3" s="215" t="s">
         <v>559</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="33" t="s">
-        <v>767</v>
-      </c>
-      <c r="B4" s="270">
+        <v>766</v>
+      </c>
+      <c r="B4" s="214">
         <v>46241</v>
       </c>
-      <c r="C4" s="270">
+      <c r="C4" s="214">
         <v>46262</v>
       </c>
-      <c r="D4" s="271" t="s">
+      <c r="D4" s="215" t="s">
         <v>559</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="33" t="s">
-        <v>768</v>
-      </c>
-      <c r="B5" s="270">
+        <v>767</v>
+      </c>
+      <c r="B5" s="214">
         <v>46262</v>
       </c>
-      <c r="C5" s="270">
+      <c r="C5" s="214">
         <v>46276</v>
       </c>
-      <c r="D5" s="271" t="s">
+      <c r="D5" s="215" t="s">
         <v>559</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="33" t="s">
-        <v>770</v>
-      </c>
-      <c r="B6" s="270">
+        <v>769</v>
+      </c>
+      <c r="B6" s="214">
         <v>46276</v>
       </c>
-      <c r="C6" s="270">
+      <c r="C6" s="214">
         <v>46283</v>
       </c>
-      <c r="D6" s="272" t="s">
-        <v>769</v>
+      <c r="D6" s="216" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="33" t="s">
-        <v>771</v>
-      </c>
-      <c r="B7" s="270">
+        <v>770</v>
+      </c>
+      <c r="B7" s="214">
         <v>46283</v>
       </c>
-      <c r="C7" s="270">
+      <c r="C7" s="214">
         <v>46290</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="33" t="s">
+        <v>771</v>
+      </c>
+      <c r="B8" s="214">
+        <v>46290</v>
+      </c>
+      <c r="C8" s="214">
+        <v>46296</v>
+      </c>
+      <c r="D8" s="33" t="s">
         <v>772</v>
-      </c>
-      <c r="B8" s="270">
-        <v>46290</v>
-      </c>
-      <c r="C8" s="270">
-        <v>46296</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="33" t="s">
-        <v>774</v>
-      </c>
-      <c r="B9" s="270">
+        <v>773</v>
+      </c>
+      <c r="B9" s="214">
         <v>46296</v>
       </c>
-      <c r="C9" s="270">
+      <c r="C9" s="214">
         <v>46311</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="33" t="s">
-        <v>775</v>
-      </c>
-      <c r="B10" s="270">
+        <v>774</v>
+      </c>
+      <c r="B10" s="214">
         <v>46311</v>
       </c>
-      <c r="C10" s="270">
+      <c r="C10" s="214">
         <v>46374</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
   </sheetData>
@@ -4672,10 +4696,10 @@
         <v>321</v>
       </c>
       <c r="B6" s="144"/>
-      <c r="C6" s="257"/>
-      <c r="D6" s="217"/>
-      <c r="E6" s="217"/>
-      <c r="F6" s="215"/>
+      <c r="C6" s="261"/>
+      <c r="D6" s="221"/>
+      <c r="E6" s="221"/>
+      <c r="F6" s="219"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" thickBot="1">
       <c r="A7" s="126" t="s">
@@ -4718,16 +4742,16 @@
       <c r="F9" s="54"/>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" thickBot="1">
-      <c r="A11" s="258" t="s">
+      <c r="A11" s="262" t="s">
         <v>329</v>
       </c>
-      <c r="B11" s="249"/>
-      <c r="C11" s="249"/>
-      <c r="D11" s="249"/>
-      <c r="E11" s="249"/>
-      <c r="F11" s="249"/>
-      <c r="G11" s="249"/>
-      <c r="H11" s="259"/>
+      <c r="B11" s="246"/>
+      <c r="C11" s="246"/>
+      <c r="D11" s="246"/>
+      <c r="E11" s="246"/>
+      <c r="F11" s="246"/>
+      <c r="G11" s="246"/>
+      <c r="H11" s="263"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" thickBot="1">
       <c r="A12" s="126" t="s">
@@ -5970,21 +5994,21 @@
   <sheetData>
     <row r="3" spans="4:10" ht="15" customHeight="1" thickBot="1"/>
     <row r="4" spans="4:10" ht="15" customHeight="1" thickBot="1">
-      <c r="D4" s="260" t="s">
+      <c r="D4" s="264" t="s">
         <v>505</v>
       </c>
-      <c r="E4" s="217"/>
-      <c r="F4" s="217"/>
-      <c r="G4" s="215"/>
+      <c r="E4" s="221"/>
+      <c r="F4" s="221"/>
+      <c r="G4" s="219"/>
     </row>
     <row r="5" spans="4:10">
-      <c r="D5" s="269" t="s">
+      <c r="D5" s="273" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="266" t="s">
+      <c r="E5" s="270" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="266" t="s">
+      <c r="F5" s="270" t="s">
         <v>506</v>
       </c>
       <c r="G5" s="49" t="s">
@@ -5992,41 +6016,41 @@
       </c>
     </row>
     <row r="6" spans="4:10">
-      <c r="D6" s="232"/>
-      <c r="E6" s="267"/>
-      <c r="F6" s="267"/>
+      <c r="D6" s="248"/>
+      <c r="E6" s="271"/>
+      <c r="F6" s="271"/>
       <c r="G6" s="51" t="s">
         <v>508</v>
       </c>
     </row>
     <row r="7" spans="4:10">
-      <c r="D7" s="232"/>
-      <c r="E7" s="267"/>
-      <c r="F7" s="267"/>
+      <c r="D7" s="248"/>
+      <c r="E7" s="271"/>
+      <c r="F7" s="271"/>
       <c r="G7" s="51" t="s">
         <v>509</v>
       </c>
     </row>
     <row r="8" spans="4:10">
-      <c r="D8" s="232"/>
-      <c r="E8" s="267"/>
-      <c r="F8" s="267"/>
+      <c r="D8" s="248"/>
+      <c r="E8" s="271"/>
+      <c r="F8" s="271"/>
       <c r="G8" s="51" t="s">
         <v>510</v>
       </c>
     </row>
     <row r="9" spans="4:10">
-      <c r="D9" s="232"/>
-      <c r="E9" s="267"/>
-      <c r="F9" s="267"/>
+      <c r="D9" s="248"/>
+      <c r="E9" s="271"/>
+      <c r="F9" s="271"/>
       <c r="G9" s="51" t="s">
         <v>460</v>
       </c>
     </row>
     <row r="10" spans="4:10">
-      <c r="D10" s="233"/>
-      <c r="E10" s="268"/>
-      <c r="F10" s="268"/>
+      <c r="D10" s="249"/>
+      <c r="E10" s="272"/>
+      <c r="F10" s="272"/>
       <c r="G10" s="51" t="s">
         <v>511</v>
       </c>
@@ -6046,19 +6070,19 @@
       <c r="E12" s="160">
         <v>1</v>
       </c>
-      <c r="F12" s="264" t="s">
+      <c r="F12" s="268" t="s">
         <v>514</v>
       </c>
-      <c r="G12" s="261" t="s">
+      <c r="G12" s="265" t="s">
         <v>515</v>
       </c>
-      <c r="H12" s="261" t="s">
+      <c r="H12" s="265" t="s">
         <v>516</v>
       </c>
-      <c r="I12" s="261" t="s">
+      <c r="I12" s="265" t="s">
         <v>517</v>
       </c>
-      <c r="J12" s="261" t="s">
+      <c r="J12" s="265" t="s">
         <v>518</v>
       </c>
     </row>
@@ -6067,22 +6091,22 @@
       <c r="E13" s="112">
         <v>2</v>
       </c>
-      <c r="F13" s="239"/>
-      <c r="G13" s="262"/>
-      <c r="H13" s="262"/>
-      <c r="I13" s="262"/>
-      <c r="J13" s="262"/>
+      <c r="F13" s="253"/>
+      <c r="G13" s="266"/>
+      <c r="H13" s="266"/>
+      <c r="I13" s="266"/>
+      <c r="J13" s="266"/>
     </row>
     <row r="14" spans="4:10" ht="15" customHeight="1" thickBot="1">
       <c r="D14" s="52"/>
       <c r="E14" s="113">
         <v>3</v>
       </c>
-      <c r="F14" s="265"/>
-      <c r="G14" s="263"/>
-      <c r="H14" s="263"/>
-      <c r="I14" s="263"/>
-      <c r="J14" s="263"/>
+      <c r="F14" s="269"/>
+      <c r="G14" s="267"/>
+      <c r="H14" s="267"/>
+      <c r="I14" s="267"/>
+      <c r="J14" s="267"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -7118,7 +7142,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9FF2DD-8784-49B6-9467-1786ED6D06B3}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C150"/>
+  <dimension ref="A1:C152"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -7754,6 +7778,9 @@
       </c>
     </row>
     <row r="58" spans="1:3" ht="86.4" hidden="1">
+      <c r="A58" t="s">
+        <v>600</v>
+      </c>
       <c r="B58" s="211" t="s">
         <v>665</v>
       </c>
@@ -7762,6 +7789,9 @@
       </c>
     </row>
     <row r="59" spans="1:3" ht="100.8" hidden="1">
+      <c r="A59" t="s">
+        <v>584</v>
+      </c>
       <c r="B59" s="211" t="s">
         <v>666</v>
       </c>
@@ -7770,6 +7800,9 @@
       </c>
     </row>
     <row r="60" spans="1:3" hidden="1">
+      <c r="A60" t="s">
+        <v>646</v>
+      </c>
       <c r="B60" s="211" t="s">
         <v>667</v>
       </c>
@@ -7778,6 +7811,9 @@
       </c>
     </row>
     <row r="61" spans="1:3" hidden="1">
+      <c r="A61" t="s">
+        <v>778</v>
+      </c>
       <c r="B61" s="211" t="s">
         <v>668</v>
       </c>
@@ -7786,6 +7822,9 @@
       </c>
     </row>
     <row r="62" spans="1:3" hidden="1">
+      <c r="A62" t="s">
+        <v>779</v>
+      </c>
       <c r="B62" s="211" t="s">
         <v>669</v>
       </c>
@@ -7794,6 +7833,9 @@
       </c>
     </row>
     <row r="63" spans="1:3" hidden="1">
+      <c r="A63" t="s">
+        <v>646</v>
+      </c>
       <c r="B63" s="211" t="s">
         <v>670</v>
       </c>
@@ -7802,6 +7844,9 @@
       </c>
     </row>
     <row r="64" spans="1:3" hidden="1">
+      <c r="A64" t="s">
+        <v>780</v>
+      </c>
       <c r="B64" s="211" t="s">
         <v>671</v>
       </c>
@@ -7809,7 +7854,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="65" spans="2:3" hidden="1">
+    <row r="65" spans="1:3" hidden="1">
+      <c r="A65" t="s">
+        <v>604</v>
+      </c>
       <c r="B65" s="211" t="s">
         <v>672</v>
       </c>
@@ -7817,7 +7865,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="66" spans="2:3" hidden="1">
+    <row r="66" spans="1:3" hidden="1">
+      <c r="A66" t="s">
+        <v>781</v>
+      </c>
       <c r="B66" s="211" t="s">
         <v>673</v>
       </c>
@@ -7825,7 +7876,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="67" spans="2:3" hidden="1">
+    <row r="67" spans="1:3" hidden="1">
+      <c r="A67" t="s">
+        <v>264</v>
+      </c>
       <c r="B67" s="211" t="s">
         <v>674</v>
       </c>
@@ -7833,7 +7887,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="68" spans="2:3" hidden="1">
+    <row r="68" spans="1:3" hidden="1">
+      <c r="A68" t="s">
+        <v>780</v>
+      </c>
       <c r="B68" s="211" t="s">
         <v>675</v>
       </c>
@@ -7841,7 +7898,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="69" spans="2:3" hidden="1">
+    <row r="69" spans="1:3" hidden="1">
+      <c r="A69" t="s">
+        <v>781</v>
+      </c>
       <c r="B69" s="211" t="s">
         <v>676</v>
       </c>
@@ -7849,7 +7909,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="70" spans="2:3" hidden="1">
+    <row r="70" spans="1:3" hidden="1">
+      <c r="A70" t="s">
+        <v>781</v>
+      </c>
       <c r="B70" s="211" t="s">
         <v>677</v>
       </c>
@@ -7857,7 +7920,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="71" spans="2:3" hidden="1">
+    <row r="71" spans="1:3" hidden="1">
+      <c r="A71" t="s">
+        <v>780</v>
+      </c>
       <c r="B71" s="211" t="s">
         <v>678</v>
       </c>
@@ -7865,7 +7931,10 @@
         <v>586</v>
       </c>
     </row>
-    <row r="72" spans="2:3" hidden="1">
+    <row r="72" spans="1:3" hidden="1">
+      <c r="A72" t="s">
+        <v>782</v>
+      </c>
       <c r="B72" s="211" t="s">
         <v>679</v>
       </c>
@@ -7873,7 +7942,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="73" spans="2:3" hidden="1">
+    <row r="73" spans="1:3">
       <c r="B73" s="211" t="s">
         <v>680</v>
       </c>
@@ -7881,7 +7950,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="74" spans="2:3" hidden="1">
+    <row r="74" spans="1:3">
       <c r="B74" s="211" t="s">
         <v>681</v>
       </c>
@@ -7889,7 +7958,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="75" spans="2:3" hidden="1">
+    <row r="75" spans="1:3">
       <c r="B75" s="211" t="s">
         <v>682</v>
       </c>
@@ -7897,7 +7966,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="76" spans="2:3" hidden="1">
+    <row r="76" spans="1:3">
       <c r="B76" s="211" t="s">
         <v>683</v>
       </c>
@@ -7905,7 +7974,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="77" spans="2:3" hidden="1">
+    <row r="77" spans="1:3">
       <c r="B77" s="211" t="s">
         <v>684</v>
       </c>
@@ -7913,7 +7982,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="78" spans="2:3" hidden="1">
+    <row r="78" spans="1:3">
       <c r="B78" s="211" t="s">
         <v>685</v>
       </c>
@@ -7921,7 +7990,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="79" spans="2:3" hidden="1">
+    <row r="79" spans="1:3">
       <c r="B79" s="211" t="s">
         <v>686</v>
       </c>
@@ -7929,7 +7998,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="80" spans="2:3" ht="28.8" hidden="1">
+    <row r="80" spans="1:3" ht="28.8">
       <c r="B80" s="211" t="s">
         <v>687</v>
       </c>
@@ -7937,7 +8006,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="81" spans="2:3" hidden="1">
+    <row r="81" spans="2:3">
       <c r="B81" s="211" t="s">
         <v>688</v>
       </c>
@@ -7945,7 +8014,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="82" spans="2:3" hidden="1">
+    <row r="82" spans="2:3">
       <c r="B82" s="211" t="s">
         <v>689</v>
       </c>
@@ -7953,7 +8022,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="83" spans="2:3" hidden="1">
+    <row r="83" spans="2:3">
       <c r="B83" s="211" t="s">
         <v>690</v>
       </c>
@@ -7961,7 +8030,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="84" spans="2:3" hidden="1">
+    <row r="84" spans="2:3">
       <c r="B84" s="211" t="s">
         <v>691</v>
       </c>
@@ -7969,7 +8038,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="85" spans="2:3" hidden="1">
+    <row r="85" spans="2:3">
       <c r="B85" s="211" t="s">
         <v>692</v>
       </c>
@@ -7977,7 +8046,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="86" spans="2:3" hidden="1">
+    <row r="86" spans="2:3">
       <c r="B86" s="211" t="s">
         <v>693</v>
       </c>
@@ -7985,7 +8054,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="87" spans="2:3" hidden="1">
+    <row r="87" spans="2:3">
       <c r="B87" s="211" t="s">
         <v>694</v>
       </c>
@@ -7993,7 +8062,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="88" spans="2:3" ht="28.8" hidden="1">
+    <row r="88" spans="2:3" ht="28.8">
       <c r="B88" s="211" t="s">
         <v>695</v>
       </c>
@@ -8001,7 +8070,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="89" spans="2:3" hidden="1">
+    <row r="89" spans="2:3">
       <c r="B89" s="211" t="s">
         <v>696</v>
       </c>
@@ -8009,7 +8078,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="90" spans="2:3" ht="28.8" hidden="1">
+    <row r="90" spans="2:3" ht="28.8">
       <c r="B90" s="211" t="s">
         <v>697</v>
       </c>
@@ -8017,7 +8086,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="91" spans="2:3" hidden="1">
+    <row r="91" spans="2:3">
       <c r="B91" s="211" t="s">
         <v>698</v>
       </c>
@@ -8025,7 +8094,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="92" spans="2:3" hidden="1">
+    <row r="92" spans="2:3">
       <c r="B92" s="211" t="s">
         <v>699</v>
       </c>
@@ -8033,7 +8102,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="93" spans="2:3" hidden="1">
+    <row r="93" spans="2:3">
       <c r="B93" s="211" t="s">
         <v>700</v>
       </c>
@@ -8041,7 +8110,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="94" spans="2:3" hidden="1">
+    <row r="94" spans="2:3">
       <c r="B94" s="211" t="s">
         <v>701</v>
       </c>
@@ -8049,7 +8118,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="95" spans="2:3" hidden="1">
+    <row r="95" spans="2:3">
       <c r="B95" s="211" t="s">
         <v>702</v>
       </c>
@@ -8057,7 +8126,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="96" spans="2:3" hidden="1">
+    <row r="96" spans="2:3">
       <c r="B96" s="213" t="s">
         <v>703</v>
       </c>
@@ -8065,7 +8134,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="97" spans="2:3" hidden="1">
+    <row r="97" spans="2:3">
       <c r="B97" s="211" t="s">
         <v>704</v>
       </c>
@@ -8073,7 +8142,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="98" spans="2:3" hidden="1">
+    <row r="98" spans="2:3">
       <c r="B98" s="211" t="s">
         <v>705</v>
       </c>
@@ -8081,7 +8150,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="99" spans="2:3" hidden="1">
+    <row r="99" spans="2:3">
       <c r="B99" s="211" t="s">
         <v>706</v>
       </c>
@@ -8089,7 +8158,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="100" spans="2:3" hidden="1">
+    <row r="100" spans="2:3">
       <c r="B100" s="211" t="s">
         <v>707</v>
       </c>
@@ -8097,7 +8166,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="101" spans="2:3" hidden="1">
+    <row r="101" spans="2:3">
       <c r="B101" s="211" t="s">
         <v>709</v>
       </c>
@@ -8105,7 +8174,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="102" spans="2:3" ht="28.8" hidden="1">
+    <row r="102" spans="2:3" ht="28.8">
       <c r="B102" s="211" t="s">
         <v>710</v>
       </c>
@@ -8113,7 +8182,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="103" spans="2:3" hidden="1">
+    <row r="103" spans="2:3">
       <c r="B103" s="211" t="s">
         <v>711</v>
       </c>
@@ -8121,7 +8190,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="104" spans="2:3" hidden="1">
+    <row r="104" spans="2:3">
       <c r="B104" s="211" t="s">
         <v>712</v>
       </c>
@@ -8129,7 +8198,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="105" spans="2:3" hidden="1">
+    <row r="105" spans="2:3">
       <c r="B105" s="211" t="s">
         <v>713</v>
       </c>
@@ -8137,7 +8206,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="106" spans="2:3" hidden="1">
+    <row r="106" spans="2:3">
       <c r="B106" s="211" t="s">
         <v>714</v>
       </c>
@@ -8145,7 +8214,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="107" spans="2:3" hidden="1">
+    <row r="107" spans="2:3">
       <c r="B107" s="211" t="s">
         <v>715</v>
       </c>
@@ -8153,7 +8222,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="108" spans="2:3" hidden="1">
+    <row r="108" spans="2:3">
       <c r="B108" s="211" t="s">
         <v>716</v>
       </c>
@@ -8161,7 +8230,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="109" spans="2:3" hidden="1">
+    <row r="109" spans="2:3">
       <c r="B109" s="211" t="s">
         <v>717</v>
       </c>
@@ -8169,7 +8238,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="110" spans="2:3" hidden="1">
+    <row r="110" spans="2:3">
       <c r="B110" s="211" t="s">
         <v>718</v>
       </c>
@@ -8177,7 +8246,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="111" spans="2:3" hidden="1">
+    <row r="111" spans="2:3">
       <c r="B111" s="211" t="s">
         <v>719</v>
       </c>
@@ -8185,7 +8254,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="112" spans="2:3" hidden="1">
+    <row r="112" spans="2:3">
       <c r="B112" s="211" t="s">
         <v>720</v>
       </c>
@@ -8193,7 +8262,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="113" spans="2:3" hidden="1">
+    <row r="113" spans="2:3">
       <c r="B113" s="211" t="s">
         <v>721</v>
       </c>
@@ -8201,7 +8270,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="114" spans="2:3" hidden="1">
+    <row r="114" spans="2:3">
       <c r="B114" s="211" t="s">
         <v>722</v>
       </c>
@@ -8209,7 +8278,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="115" spans="2:3" hidden="1">
+    <row r="115" spans="2:3">
       <c r="B115" s="211" t="s">
         <v>723</v>
       </c>
@@ -8217,7 +8286,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="116" spans="2:3" hidden="1">
+    <row r="116" spans="2:3">
       <c r="B116" s="211" t="s">
         <v>724</v>
       </c>
@@ -8225,7 +8294,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="117" spans="2:3" hidden="1">
+    <row r="117" spans="2:3">
       <c r="B117" s="211" t="s">
         <v>725</v>
       </c>
@@ -8233,7 +8302,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="118" spans="2:3" hidden="1">
+    <row r="118" spans="2:3">
       <c r="B118" s="211" t="s">
         <v>726</v>
       </c>
@@ -8241,7 +8310,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="119" spans="2:3" hidden="1">
+    <row r="119" spans="2:3">
       <c r="B119" s="211" t="s">
         <v>727</v>
       </c>
@@ -8249,7 +8318,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="120" spans="2:3" hidden="1">
+    <row r="120" spans="2:3">
       <c r="B120" s="211" t="s">
         <v>728</v>
       </c>
@@ -8257,7 +8326,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="121" spans="2:3" hidden="1">
+    <row r="121" spans="2:3">
       <c r="B121" s="211" t="s">
         <v>729</v>
       </c>
@@ -8265,7 +8334,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="122" spans="2:3" hidden="1">
+    <row r="122" spans="2:3">
       <c r="B122" s="211" t="s">
         <v>730</v>
       </c>
@@ -8273,7 +8342,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="123" spans="2:3" hidden="1">
+    <row r="123" spans="2:3">
       <c r="B123" s="211" t="s">
         <v>731</v>
       </c>
@@ -8281,7 +8350,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="124" spans="2:3" hidden="1">
+    <row r="124" spans="2:3">
       <c r="B124" s="211" t="s">
         <v>732</v>
       </c>
@@ -8289,7 +8358,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="125" spans="2:3" hidden="1">
+    <row r="125" spans="2:3">
       <c r="B125" s="211" t="s">
         <v>733</v>
       </c>
@@ -8297,15 +8366,15 @@
         <v>586</v>
       </c>
     </row>
-    <row r="126" spans="2:3" hidden="1">
+    <row r="126" spans="2:3">
       <c r="B126" s="211" t="s">
         <v>734</v>
       </c>
       <c r="C126" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="127" spans="2:3" hidden="1">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="127" spans="2:3">
       <c r="B127" s="211" t="s">
         <v>735</v>
       </c>
@@ -8313,7 +8382,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="128" spans="2:3" hidden="1">
+    <row r="128" spans="2:3">
       <c r="B128" s="211" t="s">
         <v>736</v>
       </c>
@@ -8321,7 +8390,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="129" spans="2:3" hidden="1">
+    <row r="129" spans="2:3">
       <c r="B129" s="211" t="s">
         <v>737</v>
       </c>
@@ -8329,7 +8398,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="130" spans="2:3" hidden="1">
+    <row r="130" spans="2:3">
       <c r="B130" s="211" t="s">
         <v>738</v>
       </c>
@@ -8337,7 +8406,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="131" spans="2:3" hidden="1">
+    <row r="131" spans="2:3">
       <c r="B131" s="211" t="s">
         <v>739</v>
       </c>
@@ -8345,7 +8414,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="132" spans="2:3" hidden="1">
+    <row r="132" spans="2:3">
       <c r="B132" s="211" t="s">
         <v>740</v>
       </c>
@@ -8353,7 +8422,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="133" spans="2:3" hidden="1">
+    <row r="133" spans="2:3">
       <c r="B133" s="211" t="s">
         <v>741</v>
       </c>
@@ -8361,7 +8430,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="134" spans="2:3" hidden="1">
+    <row r="134" spans="2:3">
       <c r="B134" s="211" t="s">
         <v>742</v>
       </c>
@@ -8369,7 +8438,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="135" spans="2:3" hidden="1">
+    <row r="135" spans="2:3">
       <c r="B135" s="211" t="s">
         <v>743</v>
       </c>
@@ -8377,7 +8446,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="136" spans="2:3" hidden="1">
+    <row r="136" spans="2:3">
       <c r="B136" s="211" t="s">
         <v>744</v>
       </c>
@@ -8385,7 +8454,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="137" spans="2:3" ht="28.8" hidden="1">
+    <row r="137" spans="2:3" ht="28.8">
       <c r="B137" s="211" t="s">
         <v>745</v>
       </c>
@@ -8393,7 +8462,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="138" spans="2:3" hidden="1">
+    <row r="138" spans="2:3">
       <c r="B138" s="211" t="s">
         <v>746</v>
       </c>
@@ -8401,7 +8470,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="139" spans="2:3" ht="28.8" hidden="1">
+    <row r="139" spans="2:3" ht="28.8">
       <c r="B139" s="211" t="s">
         <v>747</v>
       </c>
@@ -8409,7 +8478,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="140" spans="2:3" ht="28.8" hidden="1">
+    <row r="140" spans="2:3" ht="28.8">
       <c r="B140" s="211" t="s">
         <v>748</v>
       </c>
@@ -8417,7 +8486,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="141" spans="2:3" hidden="1">
+    <row r="141" spans="2:3">
       <c r="B141" s="211" t="s">
         <v>749</v>
       </c>
@@ -8430,10 +8499,10 @@
         <v>750</v>
       </c>
       <c r="C142" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="143" spans="2:3" hidden="1">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="143" spans="2:3">
       <c r="B143" s="211" t="s">
         <v>752</v>
       </c>
@@ -8441,7 +8510,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="144" spans="2:3" ht="28.8" hidden="1">
+    <row r="144" spans="2:3" ht="28.8">
       <c r="B144" s="211" t="s">
         <v>753</v>
       </c>
@@ -8449,7 +8518,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="145" spans="2:3" ht="28.8" hidden="1">
+    <row r="145" spans="2:3" ht="28.8">
       <c r="B145" s="211" t="s">
         <v>754</v>
       </c>
@@ -8457,7 +8526,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="146" spans="2:3" hidden="1">
+    <row r="146" spans="2:3">
       <c r="B146" s="211" t="s">
         <v>755</v>
       </c>
@@ -8470,39 +8539,53 @@
         <v>756</v>
       </c>
       <c r="C147" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="148" spans="2:3">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="148" spans="2:3" ht="28.8">
       <c r="B148" s="211" t="s">
-        <v>757</v>
+        <v>777</v>
       </c>
       <c r="C148" t="s">
-        <v>751</v>
+        <v>559</v>
       </c>
     </row>
     <row r="149" spans="2:3">
       <c r="B149" s="211" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C149" t="s">
         <v>751</v>
       </c>
     </row>
     <row r="150" spans="2:3">
-      <c r="B150" s="211" t="s">
-        <v>759</v>
+      <c r="B150" s="274" t="s">
+        <v>758</v>
       </c>
       <c r="C150" t="s">
         <v>751</v>
       </c>
     </row>
+    <row r="151" spans="2:3">
+      <c r="B151" s="211" t="s">
+        <v>775</v>
+      </c>
+      <c r="C151" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="152" spans="2:3">
+      <c r="B152" s="211" t="s">
+        <v>776</v>
+      </c>
+      <c r="C152" t="s">
+        <v>751</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C146" xr:uid="{5A64B360-020C-4527-96C0-33FA20016D59}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Pending"/>
-      </filters>
+  <autoFilter ref="A1:C152" xr:uid="{1E9FF2DD-8784-49B6-9467-1786ED6D06B3}">
+    <filterColumn colId="0">
+      <filters blank="1"/>
     </filterColumn>
   </autoFilter>
   <hyperlinks>
@@ -8532,7 +8615,7 @@
     </row>
     <row r="2" spans="2:3">
       <c r="B2" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C2" t="s">
         <v>559</v>
@@ -8540,7 +8623,7 @@
     </row>
     <row r="3" spans="2:3" ht="28.8">
       <c r="B3" s="211" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="C3" t="s">
         <v>751</v>
@@ -8639,10 +8722,10 @@
   <sheetData>
     <row r="2" spans="3:4" ht="19.05" customHeight="1" thickBot="1"/>
     <row r="3" spans="3:4" ht="19.05" customHeight="1" thickBot="1">
-      <c r="C3" s="214" t="s">
+      <c r="C3" s="218" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="215"/>
+      <c r="D3" s="219"/>
     </row>
     <row r="4" spans="3:4">
       <c r="C4" s="111" t="s">
@@ -8729,23 +8812,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="15" customHeight="1" thickBot="1">
-      <c r="B1" s="218" t="s">
+      <c r="B1" s="222" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="219"/>
-      <c r="D1" s="218" t="s">
+      <c r="C1" s="223"/>
+      <c r="D1" s="222" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="219"/>
-      <c r="F1" s="218" t="s">
+      <c r="E1" s="223"/>
+      <c r="F1" s="222" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="219"/>
-      <c r="H1" s="216" t="s">
+      <c r="G1" s="223"/>
+      <c r="H1" s="220" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="217"/>
-      <c r="J1" s="215"/>
+      <c r="I1" s="221"/>
+      <c r="J1" s="219"/>
     </row>
     <row r="2" spans="2:10">
       <c r="B2" s="11" t="s">
@@ -9156,47 +9239,47 @@
       </c>
       <c r="H2" s="88"/>
       <c r="I2" s="88"/>
-      <c r="L2" s="237" t="s">
+      <c r="L2" s="250" t="s">
         <v>114</v>
       </c>
-      <c r="M2" s="236"/>
-      <c r="N2" s="236"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
     </row>
     <row r="3" spans="2:14" s="35" customFormat="1" ht="32.1" customHeight="1">
-      <c r="B3" s="226" t="s">
+      <c r="B3" s="256" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="226" t="s">
+      <c r="C3" s="256" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="227"/>
-      <c r="E3" s="227"/>
-      <c r="F3" s="226" t="s">
+      <c r="D3" s="257"/>
+      <c r="E3" s="257"/>
+      <c r="F3" s="256" t="s">
         <v>117</v>
       </c>
       <c r="G3" s="208"/>
-      <c r="H3" s="254" t="s">
+      <c r="H3" s="239" t="s">
         <v>118</v>
       </c>
-      <c r="I3" s="255"/>
-      <c r="J3" s="238" t="s">
+      <c r="I3" s="240"/>
+      <c r="J3" s="252" t="s">
         <v>119</v>
       </c>
-      <c r="K3" s="238" t="s">
+      <c r="K3" s="252" t="s">
         <v>120</v>
       </c>
-      <c r="L3" s="224" t="s">
+      <c r="L3" s="231" t="s">
         <v>121</v>
       </c>
-      <c r="M3" s="224" t="s">
+      <c r="M3" s="231" t="s">
         <v>122</v>
       </c>
-      <c r="N3" s="224" t="s">
+      <c r="N3" s="231" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="4" spans="2:14" s="35" customFormat="1" ht="15" customHeight="1" thickBot="1">
-      <c r="B4" s="227"/>
+      <c r="B4" s="257"/>
       <c r="C4" s="210" t="s">
         <v>124</v>
       </c>
@@ -9206,15 +9289,15 @@
       <c r="E4" s="210" t="s">
         <v>126</v>
       </c>
-      <c r="F4" s="227"/>
+      <c r="F4" s="257"/>
       <c r="G4"/>
-      <c r="H4" s="256"/>
-      <c r="I4" s="225"/>
-      <c r="J4" s="239"/>
-      <c r="K4" s="239"/>
-      <c r="L4" s="225"/>
-      <c r="M4" s="225"/>
-      <c r="N4" s="225"/>
+      <c r="H4" s="241"/>
+      <c r="I4" s="232"/>
+      <c r="J4" s="253"/>
+      <c r="K4" s="253"/>
+      <c r="L4" s="232"/>
+      <c r="M4" s="232"/>
+      <c r="N4" s="232"/>
     </row>
     <row r="5" spans="2:14" s="34" customFormat="1" ht="54" customHeight="1">
       <c r="B5" s="19" t="s">
@@ -9233,10 +9316,10 @@
         <v>129</v>
       </c>
       <c r="G5" s="18"/>
-      <c r="H5" s="240" t="s">
+      <c r="H5" s="254" t="s">
         <v>130</v>
       </c>
-      <c r="I5" s="241"/>
+      <c r="I5" s="255"/>
       <c r="J5" s="137" t="s">
         <v>131</v>
       </c>
@@ -9270,10 +9353,10 @@
         <v>129</v>
       </c>
       <c r="G6" s="18"/>
-      <c r="H6" s="222" t="s">
+      <c r="H6" s="233" t="s">
         <v>136</v>
       </c>
-      <c r="I6" s="223"/>
+      <c r="I6" s="234"/>
       <c r="J6" s="138" t="s">
         <v>137</v>
       </c>
@@ -9307,10 +9390,10 @@
         <v>142</v>
       </c>
       <c r="G7" s="18"/>
-      <c r="H7" s="222" t="s">
+      <c r="H7" s="233" t="s">
         <v>143</v>
       </c>
-      <c r="I7" s="223"/>
+      <c r="I7" s="234"/>
       <c r="J7" s="138" t="s">
         <v>144</v>
       </c>
@@ -9344,10 +9427,10 @@
         <v>142</v>
       </c>
       <c r="G8" s="18"/>
-      <c r="H8" s="222" t="s">
+      <c r="H8" s="233" t="s">
         <v>149</v>
       </c>
-      <c r="I8" s="223"/>
+      <c r="I8" s="234"/>
       <c r="J8" s="138" t="s">
         <v>144</v>
       </c>
@@ -9381,10 +9464,10 @@
         <v>142</v>
       </c>
       <c r="G9" s="18"/>
-      <c r="H9" s="222" t="s">
+      <c r="H9" s="233" t="s">
         <v>154</v>
       </c>
-      <c r="I9" s="223"/>
+      <c r="I9" s="234"/>
       <c r="J9" s="138" t="s">
         <v>137</v>
       </c>
@@ -9418,10 +9501,10 @@
         <v>137</v>
       </c>
       <c r="G10" s="18"/>
-      <c r="H10" s="222" t="s">
+      <c r="H10" s="233" t="s">
         <v>159</v>
       </c>
-      <c r="I10" s="223"/>
+      <c r="I10" s="234"/>
       <c r="J10" s="138" t="s">
         <v>137</v>
       </c>
@@ -9455,10 +9538,10 @@
         <v>137</v>
       </c>
       <c r="G11" s="18"/>
-      <c r="H11" s="222" t="s">
+      <c r="H11" s="233" t="s">
         <v>165</v>
       </c>
-      <c r="I11" s="223"/>
+      <c r="I11" s="234"/>
       <c r="J11" s="138" t="s">
         <v>137</v>
       </c>
@@ -9486,10 +9569,10 @@
         <v>170</v>
       </c>
       <c r="G12" s="18"/>
-      <c r="H12" s="220" t="s">
+      <c r="H12" s="229" t="s">
         <v>171</v>
       </c>
-      <c r="I12" s="221"/>
+      <c r="I12" s="230"/>
       <c r="J12" s="139" t="s">
         <v>137</v>
       </c>
@@ -9529,8 +9612,8 @@
         <v>170</v>
       </c>
       <c r="G14" s="18"/>
-      <c r="H14" s="235"/>
-      <c r="I14" s="236"/>
+      <c r="H14" s="260"/>
+      <c r="I14" s="251"/>
       <c r="J14" s="65"/>
       <c r="K14" s="65"/>
     </row>
@@ -9934,18 +10017,18 @@
       <c r="I42" s="89"/>
     </row>
     <row r="43" spans="2:14" s="34" customFormat="1" ht="32.1" customHeight="1" thickBot="1">
-      <c r="B43" s="244" t="s">
+      <c r="B43" s="243" t="s">
         <v>203</v>
       </c>
-      <c r="C43" s="217"/>
-      <c r="D43" s="217"/>
-      <c r="E43" s="215"/>
+      <c r="C43" s="221"/>
+      <c r="D43" s="221"/>
+      <c r="E43" s="219"/>
       <c r="F43" s="18"/>
       <c r="G43" s="18"/>
-      <c r="H43" s="216" t="s">
+      <c r="H43" s="220" t="s">
         <v>118</v>
       </c>
-      <c r="I43" s="215"/>
+      <c r="I43" s="219"/>
       <c r="J43" s="141" t="s">
         <v>119</v>
       </c>
@@ -9966,14 +10049,14 @@
       <c r="C44" s="118" t="s">
         <v>116</v>
       </c>
-      <c r="D44" s="244" t="s">
+      <c r="D44" s="243" t="s">
         <v>117</v>
       </c>
-      <c r="E44" s="215"/>
-      <c r="H44" s="251" t="s">
+      <c r="E44" s="219"/>
+      <c r="H44" s="235" t="s">
         <v>205</v>
       </c>
-      <c r="I44" s="252"/>
+      <c r="I44" s="236"/>
       <c r="J44" s="142" t="s">
         <v>137</v>
       </c>
@@ -9988,7 +10071,7 @@
       </c>
     </row>
     <row r="45" spans="2:14" s="18" customFormat="1" ht="54" customHeight="1">
-      <c r="B45" s="231" t="s">
+      <c r="B45" s="237" t="s">
         <v>209</v>
       </c>
       <c r="C45" s="69" t="s">
@@ -10000,10 +10083,10 @@
       <c r="E45" s="71" t="s">
         <v>211</v>
       </c>
-      <c r="H45" s="245" t="s">
+      <c r="H45" s="225" t="s">
         <v>212</v>
       </c>
-      <c r="I45" s="246"/>
+      <c r="I45" s="226"/>
       <c r="J45" s="136" t="s">
         <v>213</v>
       </c>
@@ -10018,7 +10101,7 @@
       </c>
     </row>
     <row r="46" spans="2:14" s="18" customFormat="1" ht="54" customHeight="1">
-      <c r="B46" s="232"/>
+      <c r="B46" s="248"/>
       <c r="C46" s="67" t="s">
         <v>217</v>
       </c>
@@ -10028,10 +10111,10 @@
       <c r="E46" s="72" t="s">
         <v>211</v>
       </c>
-      <c r="H46" s="245" t="s">
+      <c r="H46" s="225" t="s">
         <v>218</v>
       </c>
-      <c r="I46" s="246"/>
+      <c r="I46" s="226"/>
       <c r="J46" s="136" t="s">
         <v>219</v>
       </c>
@@ -10046,7 +10129,7 @@
       </c>
     </row>
     <row r="47" spans="2:14" s="18" customFormat="1" ht="54" customHeight="1" thickBot="1">
-      <c r="B47" s="233"/>
+      <c r="B47" s="249"/>
       <c r="C47" s="67" t="s">
         <v>223</v>
       </c>
@@ -10056,10 +10139,10 @@
       <c r="E47" s="72" t="s">
         <v>211</v>
       </c>
-      <c r="H47" s="242" t="s">
+      <c r="H47" s="227" t="s">
         <v>224</v>
       </c>
-      <c r="I47" s="243"/>
+      <c r="I47" s="228"/>
       <c r="J47" s="85" t="s">
         <v>225</v>
       </c>
@@ -10197,7 +10280,7 @@
         <v>170</v>
       </c>
       <c r="E57" s="25"/>
-      <c r="H57" s="228" t="s">
+      <c r="H57" s="258" t="s">
         <v>236</v>
       </c>
       <c r="I57" s="91" t="s">
@@ -10217,7 +10300,7 @@
       </c>
     </row>
     <row r="58" spans="2:15" s="18" customFormat="1" ht="14.55" customHeight="1">
-      <c r="B58" s="234" t="s">
+      <c r="B58" s="247" t="s">
         <v>242</v>
       </c>
       <c r="C58" s="46" t="s">
@@ -10226,7 +10309,7 @@
       <c r="D58" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="H58" s="229"/>
+      <c r="H58" s="245"/>
       <c r="I58" s="92" t="s">
         <v>244</v>
       </c>
@@ -10235,14 +10318,14 @@
       </c>
     </row>
     <row r="59" spans="2:15" s="18" customFormat="1" ht="14.55" customHeight="1">
-      <c r="B59" s="232"/>
+      <c r="B59" s="248"/>
       <c r="C59" s="46" t="s">
         <v>244</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="H59" s="229"/>
+      <c r="H59" s="245"/>
       <c r="I59" s="92" t="s">
         <v>245</v>
       </c>
@@ -10251,14 +10334,14 @@
       </c>
     </row>
     <row r="60" spans="2:15" s="18" customFormat="1" ht="14.55" customHeight="1">
-      <c r="B60" s="232"/>
+      <c r="B60" s="248"/>
       <c r="C60" s="46" t="s">
         <v>245</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="H60" s="230"/>
+      <c r="H60" s="259"/>
       <c r="I60" s="92" t="s">
         <v>246</v>
       </c>
@@ -10267,7 +10350,7 @@
       </c>
     </row>
     <row r="61" spans="2:15" s="18" customFormat="1" ht="54" customHeight="1">
-      <c r="B61" s="233"/>
+      <c r="B61" s="249"/>
       <c r="C61" s="46" t="s">
         <v>246</v>
       </c>
@@ -10328,7 +10411,7 @@
       <c r="D63" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="H63" s="248" t="s">
+      <c r="H63" s="244" t="s">
         <v>257</v>
       </c>
       <c r="I63" s="92" t="s">
@@ -10357,7 +10440,7 @@
       <c r="D64" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="H64" s="229"/>
+      <c r="H64" s="245"/>
       <c r="I64" s="92" t="s">
         <v>244</v>
       </c>
@@ -10375,7 +10458,7 @@
       <c r="D65" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="H65" s="229"/>
+      <c r="H65" s="245"/>
       <c r="I65" s="92" t="s">
         <v>245</v>
       </c>
@@ -10384,7 +10467,7 @@
       </c>
     </row>
     <row r="66" spans="2:14" s="18" customFormat="1" ht="15" customHeight="1" thickBot="1">
-      <c r="B66" s="234" t="s">
+      <c r="B66" s="247" t="s">
         <v>257</v>
       </c>
       <c r="C66" s="46" t="s">
@@ -10393,7 +10476,7 @@
       <c r="D66" s="21" t="s">
         <v>263</v>
       </c>
-      <c r="H66" s="249"/>
+      <c r="H66" s="246"/>
       <c r="I66" s="93" t="s">
         <v>246</v>
       </c>
@@ -10402,7 +10485,7 @@
       </c>
     </row>
     <row r="67" spans="2:14" s="18" customFormat="1" ht="14.55" customHeight="1">
-      <c r="B67" s="232"/>
+      <c r="B67" s="248"/>
       <c r="C67" s="46" t="s">
         <v>244</v>
       </c>
@@ -10413,7 +10496,7 @@
       <c r="I67" s="66"/>
     </row>
     <row r="68" spans="2:14" s="18" customFormat="1" ht="14.55" customHeight="1">
-      <c r="B68" s="232"/>
+      <c r="B68" s="248"/>
       <c r="C68" s="46" t="s">
         <v>245</v>
       </c>
@@ -10424,7 +10507,7 @@
       <c r="I68" s="66"/>
     </row>
     <row r="69" spans="2:14" s="18" customFormat="1" ht="15" customHeight="1" thickBot="1">
-      <c r="B69" s="233"/>
+      <c r="B69" s="249"/>
       <c r="C69" s="73" t="s">
         <v>246</v>
       </c>
@@ -10451,10 +10534,10 @@
       <c r="C73" s="124" t="s">
         <v>119</v>
       </c>
-      <c r="H73" s="247" t="s">
+      <c r="H73" s="242" t="s">
         <v>265</v>
       </c>
-      <c r="I73" s="219"/>
+      <c r="I73" s="223"/>
       <c r="J73" s="125" t="s">
         <v>119</v>
       </c>
@@ -10475,10 +10558,10 @@
       <c r="C74" s="70" t="s">
         <v>170</v>
       </c>
-      <c r="H74" s="231" t="s">
+      <c r="H74" s="237" t="s">
         <v>165</v>
       </c>
-      <c r="I74" s="253"/>
+      <c r="I74" s="238"/>
       <c r="J74" s="45" t="s">
         <v>137</v>
       </c>
@@ -10499,10 +10582,10 @@
       <c r="C75" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="H75" s="222" t="s">
+      <c r="H75" s="233" t="s">
         <v>171</v>
       </c>
-      <c r="I75" s="223"/>
+      <c r="I75" s="234"/>
       <c r="J75" s="21" t="s">
         <v>137</v>
       </c>
@@ -10523,10 +10606,10 @@
       <c r="C76" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="H76" s="222" t="s">
+      <c r="H76" s="233" t="s">
         <v>270</v>
       </c>
-      <c r="I76" s="223"/>
+      <c r="I76" s="234"/>
       <c r="J76" s="21" t="s">
         <v>137</v>
       </c>
@@ -10547,10 +10630,10 @@
       <c r="C77" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="H77" s="222" t="s">
+      <c r="H77" s="233" t="s">
         <v>275</v>
       </c>
-      <c r="I77" s="223"/>
+      <c r="I77" s="234"/>
       <c r="J77" s="21" t="s">
         <v>276</v>
       </c>
@@ -10571,10 +10654,10 @@
       <c r="C78" s="68" t="s">
         <v>263</v>
       </c>
-      <c r="H78" s="220" t="s">
+      <c r="H78" s="229" t="s">
         <v>281</v>
       </c>
-      <c r="I78" s="221"/>
+      <c r="I78" s="230"/>
       <c r="J78" s="24" t="s">
         <v>282</v>
       </c>
@@ -10615,10 +10698,10 @@
       <c r="C83" s="124" t="s">
         <v>119</v>
       </c>
-      <c r="H83" s="247" t="s">
+      <c r="H83" s="242" t="s">
         <v>118</v>
       </c>
-      <c r="I83" s="219"/>
+      <c r="I83" s="223"/>
       <c r="J83" s="122" t="s">
         <v>119</v>
       </c>
@@ -10639,10 +10722,10 @@
       <c r="C84" s="70" t="s">
         <v>263</v>
       </c>
-      <c r="H84" s="231" t="s">
+      <c r="H84" s="237" t="s">
         <v>289</v>
       </c>
-      <c r="I84" s="253"/>
+      <c r="I84" s="238"/>
       <c r="J84" s="74" t="s">
         <v>137</v>
       </c>
@@ -10663,10 +10746,10 @@
       <c r="C85" s="68" t="s">
         <v>263</v>
       </c>
-      <c r="H85" s="220" t="s">
+      <c r="H85" s="229" t="s">
         <v>294</v>
       </c>
-      <c r="I85" s="221"/>
+      <c r="I85" s="230"/>
       <c r="J85" s="24" t="s">
         <v>137</v>
       </c>
@@ -10710,10 +10793,10 @@
       <c r="C89" s="124" t="s">
         <v>234</v>
       </c>
-      <c r="H89" s="247" t="s">
+      <c r="H89" s="242" t="s">
         <v>118</v>
       </c>
-      <c r="I89" s="219"/>
+      <c r="I89" s="223"/>
       <c r="J89" s="122" t="s">
         <v>119</v>
       </c>
@@ -10734,10 +10817,10 @@
       <c r="C90" s="81" t="s">
         <v>170</v>
       </c>
-      <c r="H90" s="251" t="s">
+      <c r="H90" s="235" t="s">
         <v>301</v>
       </c>
-      <c r="I90" s="252"/>
+      <c r="I90" s="236"/>
       <c r="J90" s="83" t="s">
         <v>137</v>
       </c>
@@ -10758,10 +10841,10 @@
       <c r="C91" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="H91" s="245" t="s">
+      <c r="H91" s="225" t="s">
         <v>306</v>
       </c>
-      <c r="I91" s="246"/>
+      <c r="I91" s="226"/>
       <c r="J91" s="84" t="s">
         <v>137</v>
       </c>
@@ -10782,10 +10865,10 @@
       <c r="C92" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="H92" s="242" t="s">
+      <c r="H92" s="227" t="s">
         <v>311</v>
       </c>
-      <c r="I92" s="243"/>
+      <c r="I92" s="228"/>
       <c r="J92" s="82" t="s">
         <v>243</v>
       </c>
@@ -10829,10 +10912,10 @@
       <c r="L96" s="200" t="s">
         <v>319</v>
       </c>
-      <c r="M96" s="250" t="s">
+      <c r="M96" s="224" t="s">
         <v>320</v>
       </c>
-      <c r="N96" s="250"/>
+      <c r="N96" s="224"/>
     </row>
     <row r="97" s="18" customFormat="1" ht="14.55" customHeight="1"/>
     <row r="98" s="18" customFormat="1" ht="14.55" customHeight="1"/>
@@ -10853,6 +10936,35 @@
     <row r="113" s="18" customFormat="1" ht="14.55" customHeight="1"/>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H77:I77"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H57:H60"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="H92:I92"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="H89:I89"/>
+    <mergeCell ref="H63:H66"/>
+    <mergeCell ref="H73:I73"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="H43:I43"/>
     <mergeCell ref="M96:N96"/>
     <mergeCell ref="H91:I91"/>
     <mergeCell ref="H47:I47"/>
@@ -10869,35 +10981,6 @@
     <mergeCell ref="H78:I78"/>
     <mergeCell ref="H74:I74"/>
     <mergeCell ref="H83:I83"/>
-    <mergeCell ref="H92:I92"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="H89:I89"/>
-    <mergeCell ref="H63:H66"/>
-    <mergeCell ref="H73:I73"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H77:I77"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H57:H60"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="H14:I14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>